<commit_message>
docs: update documentation, regenerate example reports, and achieve 10/10 pylint
</commit_message>
<xml_diff>
--- a/examples/dual_isotope_water/Synthetic_Water_18O_Report.xlsx
+++ b/examples/dual_isotope_water/Synthetic_Water_18O_Report.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="Results" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Parameters" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Uncertainty_Budget" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Parameters" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -449,7 +450,7 @@
         <v>-12.55</v>
       </c>
       <c r="C2" t="n">
-        <v>0.16</v>
+        <v>0.26</v>
       </c>
       <c r="D2" t="n">
         <v>4</v>
@@ -465,7 +466,7 @@
         <v>-5.9</v>
       </c>
       <c r="C3" t="n">
-        <v>0.12</v>
+        <v>0.24</v>
       </c>
       <c r="D3" t="n">
         <v>6</v>
@@ -481,7 +482,7 @@
         <v>0.24</v>
       </c>
       <c r="C4" t="n">
-        <v>0.21</v>
+        <v>0.29</v>
       </c>
       <c r="D4" t="n">
         <v>4</v>
@@ -497,7 +498,7 @@
         <v>-11.4</v>
       </c>
       <c r="C5" t="n">
-        <v>0.14</v>
+        <v>0.25</v>
       </c>
       <c r="D5" t="n">
         <v>4</v>
@@ -513,7 +514,7 @@
         <v>-3.02</v>
       </c>
       <c r="C6" t="n">
-        <v>0.19</v>
+        <v>0.28</v>
       </c>
       <c r="D6" t="n">
         <v>2</v>
@@ -529,7 +530,7 @@
         <v>-4.39</v>
       </c>
       <c r="C7" t="n">
-        <v>0.27</v>
+        <v>0.34</v>
       </c>
       <c r="D7" t="n">
         <v>1</v>
@@ -545,7 +546,7 @@
         <v>-1.98</v>
       </c>
       <c r="C8" t="n">
-        <v>0.18</v>
+        <v>0.28</v>
       </c>
       <c r="D8" t="n">
         <v>2</v>
@@ -561,7 +562,7 @@
         <v>-4.95</v>
       </c>
       <c r="C9" t="n">
-        <v>0.13</v>
+        <v>0.24</v>
       </c>
       <c r="D9" t="n">
         <v>2</v>
@@ -577,7 +578,7 @@
         <v>-6.85</v>
       </c>
       <c r="C10" t="n">
-        <v>0.14</v>
+        <v>0.25</v>
       </c>
       <c r="D10" t="n">
         <v>2</v>
@@ -593,7 +594,7 @@
         <v>-7.49</v>
       </c>
       <c r="C11" t="n">
-        <v>0.11</v>
+        <v>0.24</v>
       </c>
       <c r="D11" t="n">
         <v>2</v>
@@ -609,7 +610,7 @@
         <v>-9.19</v>
       </c>
       <c r="C12" t="n">
-        <v>0.16</v>
+        <v>0.26</v>
       </c>
       <c r="D12" t="n">
         <v>2</v>
@@ -625,7 +626,7 @@
         <v>-10.97</v>
       </c>
       <c r="C13" t="n">
-        <v>0.14</v>
+        <v>0.25</v>
       </c>
       <c r="D13" t="n">
         <v>2</v>
@@ -642,7 +643,399 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:H13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>group_name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>combined_uncertainty</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>pct_measurement</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>pct_anchors</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>pct_fit_residual</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>pct_blank</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>pct_linearity</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>pct_drift</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Antartida_O</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="D2" t="n">
+        <v>36.27</v>
+      </c>
+      <c r="E2" t="n">
+        <v>63.08</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Buenos Aires_O</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="D3" t="n">
+        <v>24.06</v>
+      </c>
+      <c r="E3" t="n">
+        <v>74.7</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Mar_O</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="C4" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="D4" t="n">
+        <v>48.35</v>
+      </c>
+      <c r="E4" t="n">
+        <v>49.26</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Mendoza_O</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C5" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="D5" t="n">
+        <v>30.73</v>
+      </c>
+      <c r="E5" t="n">
+        <v>66.91</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Rain_Water_01</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="C6" t="n">
+        <v>18.56</v>
+      </c>
+      <c r="D6" t="n">
+        <v>27.97</v>
+      </c>
+      <c r="E6" t="n">
+        <v>53.29</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Rain_Water_02</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="C7" t="n">
+        <v>49.14</v>
+      </c>
+      <c r="D7" t="n">
+        <v>14.65</v>
+      </c>
+      <c r="E7" t="n">
+        <v>36.16</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Rain_Water_03</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="C8" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="D8" t="n">
+        <v>35.93</v>
+      </c>
+      <c r="E8" t="n">
+        <v>55.75</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.42</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Rain_Water_04</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="D9" t="n">
+        <v>26.25</v>
+      </c>
+      <c r="E9" t="n">
+        <v>71.34</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>River_Water_01</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C10" t="n">
+        <v>10.22</v>
+      </c>
+      <c r="D10" t="n">
+        <v>20.34</v>
+      </c>
+      <c r="E10" t="n">
+        <v>68.52</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.91</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>River_Water_02</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="D11" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="E11" t="n">
+        <v>76.23</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.57</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>River_Water_03</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="C12" t="n">
+        <v>17.23</v>
+      </c>
+      <c r="D12" t="n">
+        <v>20.13</v>
+      </c>
+      <c r="E12" t="n">
+        <v>62.59</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>River_Water_04</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="D13" t="n">
+        <v>29.41</v>
+      </c>
+      <c r="E13" t="n">
+        <v>69.37</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.23</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -667,119 +1060,119 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Strategy</t>
+          <t>International Scale</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>MultiPointLinear</t>
+          <t>VSMOW-SLAP</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Target Column</t>
+          <t>Strategy</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>d18o</t>
+          <t>MultiPointLinear</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Filepath</t>
+          <t>Target Column</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>/home/damm/Projects/isotools/examples/dual_isotope_water/synthetic_water_sequence.xlsx</t>
+          <t>d18o</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Anchors</t>
+          <t>Filepath</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Mar_O, Buenos Aires_O, Mendoza_O, Antartida_O</t>
+          <t>/home/damm/Projects/isotools/examples/dual_isotope_water/synthetic_water_sequence.xlsx</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Controls</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
+          <t>Anchors</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Mar_O, Buenos Aires_O, Mendoza_O, Antartida_O</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Drift Monitors</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Buenos Aires_O</t>
-        </is>
-      </c>
+          <t>Controls</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Blank Correction Applied</t>
-        </is>
-      </c>
-      <c r="B9" t="b">
-        <v>0</v>
+          <t>Drift Monitors</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Buenos Aires_O</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Blank Identifier</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
+          <t>Memory Correction Applied</t>
+        </is>
+      </c>
+      <c r="B10" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Linearity Correction Applied</t>
-        </is>
-      </c>
-      <c r="B11" t="b">
-        <v>0</v>
+          <t>Memory Coefficients</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Linearity Slope</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
+          <t>Blank Correction Applied</t>
+        </is>
+      </c>
+      <c r="B12" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Linearity Slope 95% CI</t>
+          <t>Blank Identifier</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -791,19 +1184,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Linearity Slope Source</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
+          <t>Linearity Correction Applied</t>
+        </is>
+      </c>
+      <c r="B14" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Linearity Reference Substance</t>
+          <t>Linearity Slope</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -815,7 +1206,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Linearity Ref Area</t>
+          <t>Linearity Slope 95% CI</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -827,62 +1218,118 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Drift Correction Applied</t>
-        </is>
-      </c>
-      <c r="B17" t="b">
-        <v>1</v>
+          <t>Linearity Slope Source</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Drift Monitor Used</t>
+          <t>Linearity Reference Substance</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Buenos Aires_O</t>
+          <t>None</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Drift Slope</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>0.01001315413211323</v>
+          <t>Linearity Ref Area</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Drift Slope 95% CI</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>0.008244994178859972</v>
+          <t>Drift Correction Applied</t>
+        </is>
+      </c>
+      <c r="B20" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Slope</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>0.998745895715564</v>
+          <t>Drift Monitor Used</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Buenos Aires_O</t>
+        </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>Drift Polynomial Degree</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Drift Slope</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>0.01001315413211323</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Drift Slope 95% CI</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>0.008244994178859972</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Elemental Calibration Applied</t>
+        </is>
+      </c>
+      <c r="B25" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Slope</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>0.998745895715564</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>Intercept</t>
         </is>
       </c>
-      <c r="B22" t="n">
+      <c r="B27" t="n">
         <v>-1.459682876825608</v>
       </c>
     </row>

</xml_diff>